<commit_message>
adjusted building material calculation
</commit_message>
<xml_diff>
--- a/data_input/MI_Buildings_Oorschot2023.xlsx
+++ b/data_input/MI_Buildings_Oorschot2023.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Mira/Documents/IE/REAL UTOPIAN HOUSING/Post-GrowthHousingScenarios/Code/housing-footprints/data_input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C266CA18-0F84-B645-8ED8-B1CC5C1D3A29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6A3E593-33EB-4540-B39B-01C96BD18665}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10660" yWindow="500" windowWidth="14940" windowHeight="15500" tabRatio="902" activeTab="2" xr2:uid="{501A363E-84AB-4328-B285-EDCE5CC29F1E}"/>
   </bookViews>
@@ -2139,9 +2139,6 @@
     <t>1975-2005</t>
   </si>
   <si>
-    <t>2006-2018</t>
-  </si>
-  <si>
     <t>pre 1945</t>
   </si>
   <si>
@@ -2155,6 +2152,9 @@
   </si>
   <si>
     <t>multiple fam (meergezins)</t>
+  </si>
+  <si>
+    <t>2006-2022</t>
   </si>
 </sst>
 </file>
@@ -4432,16 +4432,10 @@
     <xf numFmtId="0" fontId="57" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -4450,7 +4444,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -21200,11 +21200,11 @@
       </c>
     </row>
     <row r="2" spans="1:18" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="571">
+      <c r="A2" s="575">
         <v>2018</v>
       </c>
-      <c r="B2" s="572"/>
-      <c r="C2" s="572"/>
+      <c r="B2" s="576"/>
+      <c r="C2" s="576"/>
       <c r="D2" s="174">
         <v>1849352203.1438973</v>
       </c>
@@ -21248,10 +21248,10 @@
       <c r="R2" s="175"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A3" s="573" t="s">
+      <c r="A3" s="577" t="s">
         <v>235</v>
       </c>
-      <c r="B3" s="575" t="s">
+      <c r="B3" s="573" t="s">
         <v>271</v>
       </c>
       <c r="C3" s="37" t="s">
@@ -21304,8 +21304,8 @@
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A4" s="574"/>
-      <c r="B4" s="576"/>
+      <c r="A4" s="571"/>
+      <c r="B4" s="574"/>
       <c r="C4" s="11" t="s">
         <v>272</v>
       </c>
@@ -21356,8 +21356,8 @@
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A5" s="574"/>
-      <c r="B5" s="576"/>
+      <c r="A5" s="571"/>
+      <c r="B5" s="574"/>
       <c r="C5" s="11" t="s">
         <v>273</v>
       </c>
@@ -21408,8 +21408,8 @@
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A6" s="574"/>
-      <c r="B6" s="576" t="s">
+      <c r="A6" s="571"/>
+      <c r="B6" s="574" t="s">
         <v>274</v>
       </c>
       <c r="C6" s="11" t="s">
@@ -21462,8 +21462,8 @@
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A7" s="574"/>
-      <c r="B7" s="576"/>
+      <c r="A7" s="571"/>
+      <c r="B7" s="574"/>
       <c r="C7" s="11" t="s">
         <v>272</v>
       </c>
@@ -21514,8 +21514,8 @@
       </c>
     </row>
     <row r="8" spans="1:18" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="574"/>
-      <c r="B8" s="576"/>
+      <c r="A8" s="571"/>
+      <c r="B8" s="574"/>
       <c r="C8" s="11" t="s">
         <v>273</v>
       </c>
@@ -21566,10 +21566,10 @@
       </c>
     </row>
     <row r="9" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="574" t="s">
+      <c r="A9" s="571" t="s">
         <v>275</v>
       </c>
-      <c r="B9" s="575" t="s">
+      <c r="B9" s="573" t="s">
         <v>271</v>
       </c>
       <c r="C9" s="37" t="s">
@@ -21622,8 +21622,8 @@
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A10" s="574"/>
-      <c r="B10" s="576"/>
+      <c r="A10" s="571"/>
+      <c r="B10" s="574"/>
       <c r="C10" s="11" t="s">
         <v>272</v>
       </c>
@@ -21674,8 +21674,8 @@
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A11" s="574"/>
-      <c r="B11" s="576"/>
+      <c r="A11" s="571"/>
+      <c r="B11" s="574"/>
       <c r="C11" s="11" t="s">
         <v>273</v>
       </c>
@@ -21726,8 +21726,8 @@
       </c>
     </row>
     <row r="12" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="574"/>
-      <c r="B12" s="576" t="s">
+      <c r="A12" s="571"/>
+      <c r="B12" s="574" t="s">
         <v>274</v>
       </c>
       <c r="C12" s="11" t="s">
@@ -21780,8 +21780,8 @@
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A13" s="574"/>
-      <c r="B13" s="576"/>
+      <c r="A13" s="571"/>
+      <c r="B13" s="574"/>
       <c r="C13" s="11" t="s">
         <v>272</v>
       </c>
@@ -21832,8 +21832,8 @@
       </c>
     </row>
     <row r="14" spans="1:18" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="574"/>
-      <c r="B14" s="576"/>
+      <c r="A14" s="571"/>
+      <c r="B14" s="574"/>
       <c r="C14" s="11" t="s">
         <v>273</v>
       </c>
@@ -21884,10 +21884,10 @@
       </c>
     </row>
     <row r="15" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="574" t="s">
+      <c r="A15" s="571" t="s">
         <v>276</v>
       </c>
-      <c r="B15" s="575" t="s">
+      <c r="B15" s="573" t="s">
         <v>271</v>
       </c>
       <c r="C15" s="37" t="s">
@@ -21940,8 +21940,8 @@
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A16" s="574"/>
-      <c r="B16" s="576"/>
+      <c r="A16" s="571"/>
+      <c r="B16" s="574"/>
       <c r="C16" s="11" t="s">
         <v>272</v>
       </c>
@@ -21992,8 +21992,8 @@
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A17" s="574"/>
-      <c r="B17" s="576"/>
+      <c r="A17" s="571"/>
+      <c r="B17" s="574"/>
       <c r="C17" s="11" t="s">
         <v>273</v>
       </c>
@@ -22044,8 +22044,8 @@
       </c>
     </row>
     <row r="18" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="574"/>
-      <c r="B18" s="576" t="s">
+      <c r="A18" s="571"/>
+      <c r="B18" s="574" t="s">
         <v>274</v>
       </c>
       <c r="C18" s="11" t="s">
@@ -22098,8 +22098,8 @@
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A19" s="574"/>
-      <c r="B19" s="576"/>
+      <c r="A19" s="571"/>
+      <c r="B19" s="574"/>
       <c r="C19" s="11" t="s">
         <v>272</v>
       </c>
@@ -22150,8 +22150,8 @@
       </c>
     </row>
     <row r="20" spans="1:18" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="574"/>
-      <c r="B20" s="576"/>
+      <c r="A20" s="571"/>
+      <c r="B20" s="574"/>
       <c r="C20" s="11" t="s">
         <v>273</v>
       </c>
@@ -22202,10 +22202,10 @@
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A21" s="574" t="s">
+      <c r="A21" s="571" t="s">
         <v>236</v>
       </c>
-      <c r="B21" s="575" t="s">
+      <c r="B21" s="573" t="s">
         <v>271</v>
       </c>
       <c r="C21" s="37" t="s">
@@ -22258,8 +22258,8 @@
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A22" s="574"/>
-      <c r="B22" s="576"/>
+      <c r="A22" s="571"/>
+      <c r="B22" s="574"/>
       <c r="C22" s="11" t="s">
         <v>272</v>
       </c>
@@ -22310,8 +22310,8 @@
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A23" s="574"/>
-      <c r="B23" s="576"/>
+      <c r="A23" s="571"/>
+      <c r="B23" s="574"/>
       <c r="C23" s="11" t="s">
         <v>273</v>
       </c>
@@ -22362,8 +22362,8 @@
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A24" s="574"/>
-      <c r="B24" s="576" t="s">
+      <c r="A24" s="571"/>
+      <c r="B24" s="574" t="s">
         <v>274</v>
       </c>
       <c r="C24" s="11" t="s">
@@ -22416,8 +22416,8 @@
       </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A25" s="574"/>
-      <c r="B25" s="576"/>
+      <c r="A25" s="571"/>
+      <c r="B25" s="574"/>
       <c r="C25" s="11" t="s">
         <v>272</v>
       </c>
@@ -22468,8 +22468,8 @@
       </c>
     </row>
     <row r="26" spans="1:18" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="574"/>
-      <c r="B26" s="576"/>
+      <c r="A26" s="571"/>
+      <c r="B26" s="574"/>
       <c r="C26" s="11" t="s">
         <v>273</v>
       </c>
@@ -22520,10 +22520,10 @@
       </c>
     </row>
     <row r="27" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="574" t="s">
+      <c r="A27" s="571" t="s">
         <v>277</v>
       </c>
-      <c r="B27" s="575" t="s">
+      <c r="B27" s="573" t="s">
         <v>271</v>
       </c>
       <c r="C27" s="37" t="s">
@@ -22576,8 +22576,8 @@
       </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A28" s="574"/>
-      <c r="B28" s="576"/>
+      <c r="A28" s="571"/>
+      <c r="B28" s="574"/>
       <c r="C28" s="11" t="s">
         <v>272</v>
       </c>
@@ -22628,8 +22628,8 @@
       </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A29" s="574"/>
-      <c r="B29" s="576"/>
+      <c r="A29" s="571"/>
+      <c r="B29" s="574"/>
       <c r="C29" s="11" t="s">
         <v>273</v>
       </c>
@@ -22680,8 +22680,8 @@
       </c>
     </row>
     <row r="30" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="574"/>
-      <c r="B30" s="576" t="s">
+      <c r="A30" s="571"/>
+      <c r="B30" s="574" t="s">
         <v>274</v>
       </c>
       <c r="C30" s="11" t="s">
@@ -22734,8 +22734,8 @@
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A31" s="574"/>
-      <c r="B31" s="576"/>
+      <c r="A31" s="571"/>
+      <c r="B31" s="574"/>
       <c r="C31" s="11" t="s">
         <v>272</v>
       </c>
@@ -22786,8 +22786,8 @@
       </c>
     </row>
     <row r="32" spans="1:18" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="574"/>
-      <c r="B32" s="576"/>
+      <c r="A32" s="571"/>
+      <c r="B32" s="574"/>
       <c r="C32" s="11" t="s">
         <v>273</v>
       </c>
@@ -22838,10 +22838,10 @@
       </c>
     </row>
     <row r="33" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="574" t="s">
+      <c r="A33" s="571" t="s">
         <v>278</v>
       </c>
-      <c r="B33" s="575" t="s">
+      <c r="B33" s="573" t="s">
         <v>271</v>
       </c>
       <c r="C33" s="37" t="s">
@@ -22894,8 +22894,8 @@
       </c>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A34" s="574"/>
-      <c r="B34" s="576"/>
+      <c r="A34" s="571"/>
+      <c r="B34" s="574"/>
       <c r="C34" s="11" t="s">
         <v>272</v>
       </c>
@@ -22946,8 +22946,8 @@
       </c>
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A35" s="574"/>
-      <c r="B35" s="576"/>
+      <c r="A35" s="571"/>
+      <c r="B35" s="574"/>
       <c r="C35" s="11" t="s">
         <v>273</v>
       </c>
@@ -22998,8 +22998,8 @@
       </c>
     </row>
     <row r="36" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="574"/>
-      <c r="B36" s="576" t="s">
+      <c r="A36" s="571"/>
+      <c r="B36" s="574" t="s">
         <v>274</v>
       </c>
       <c r="C36" s="11" t="s">
@@ -23052,8 +23052,8 @@
       </c>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A37" s="574"/>
-      <c r="B37" s="576"/>
+      <c r="A37" s="571"/>
+      <c r="B37" s="574"/>
       <c r="C37" s="11" t="s">
         <v>272</v>
       </c>
@@ -23104,8 +23104,8 @@
       </c>
     </row>
     <row r="38" spans="1:18" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="574"/>
-      <c r="B38" s="576"/>
+      <c r="A38" s="571"/>
+      <c r="B38" s="574"/>
       <c r="C38" s="11" t="s">
         <v>273</v>
       </c>
@@ -23156,10 +23156,10 @@
       </c>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A39" s="574" t="s">
+      <c r="A39" s="571" t="s">
         <v>241</v>
       </c>
-      <c r="B39" s="575" t="s">
+      <c r="B39" s="573" t="s">
         <v>271</v>
       </c>
       <c r="C39" s="37" t="s">
@@ -23212,8 +23212,8 @@
       </c>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A40" s="574"/>
-      <c r="B40" s="576"/>
+      <c r="A40" s="571"/>
+      <c r="B40" s="574"/>
       <c r="C40" s="11" t="s">
         <v>272</v>
       </c>
@@ -23264,8 +23264,8 @@
       </c>
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A41" s="574"/>
-      <c r="B41" s="576"/>
+      <c r="A41" s="571"/>
+      <c r="B41" s="574"/>
       <c r="C41" s="11" t="s">
         <v>273</v>
       </c>
@@ -23316,8 +23316,8 @@
       </c>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A42" s="574"/>
-      <c r="B42" s="576" t="s">
+      <c r="A42" s="571"/>
+      <c r="B42" s="574" t="s">
         <v>274</v>
       </c>
       <c r="C42" s="11" t="s">
@@ -23370,8 +23370,8 @@
       </c>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A43" s="574"/>
-      <c r="B43" s="576"/>
+      <c r="A43" s="571"/>
+      <c r="B43" s="574"/>
       <c r="C43" s="11" t="s">
         <v>272</v>
       </c>
@@ -23422,8 +23422,8 @@
       </c>
     </row>
     <row r="44" spans="1:18" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="574"/>
-      <c r="B44" s="576"/>
+      <c r="A44" s="571"/>
+      <c r="B44" s="574"/>
       <c r="C44" s="11" t="s">
         <v>273</v>
       </c>
@@ -23474,10 +23474,10 @@
       </c>
     </row>
     <row r="45" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="574" t="s">
+      <c r="A45" s="571" t="s">
         <v>393</v>
       </c>
-      <c r="B45" s="575" t="s">
+      <c r="B45" s="573" t="s">
         <v>271</v>
       </c>
       <c r="C45" s="37" t="s">
@@ -23530,8 +23530,8 @@
       </c>
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A46" s="574"/>
-      <c r="B46" s="576"/>
+      <c r="A46" s="571"/>
+      <c r="B46" s="574"/>
       <c r="C46" s="11" t="s">
         <v>272</v>
       </c>
@@ -23582,8 +23582,8 @@
       </c>
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A47" s="574"/>
-      <c r="B47" s="576"/>
+      <c r="A47" s="571"/>
+      <c r="B47" s="574"/>
       <c r="C47" s="11" t="s">
         <v>273</v>
       </c>
@@ -23634,8 +23634,8 @@
       </c>
     </row>
     <row r="48" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="574"/>
-      <c r="B48" s="576" t="s">
+      <c r="A48" s="571"/>
+      <c r="B48" s="574" t="s">
         <v>274</v>
       </c>
       <c r="C48" s="11" t="s">
@@ -23688,8 +23688,8 @@
       </c>
     </row>
     <row r="49" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A49" s="574"/>
-      <c r="B49" s="576"/>
+      <c r="A49" s="571"/>
+      <c r="B49" s="574"/>
       <c r="C49" s="11" t="s">
         <v>272</v>
       </c>
@@ -23740,8 +23740,8 @@
       </c>
     </row>
     <row r="50" spans="1:18" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="574"/>
-      <c r="B50" s="576"/>
+      <c r="A50" s="571"/>
+      <c r="B50" s="574"/>
       <c r="C50" s="11" t="s">
         <v>273</v>
       </c>
@@ -23792,10 +23792,10 @@
       </c>
     </row>
     <row r="51" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="574" t="s">
+      <c r="A51" s="571" t="s">
         <v>394</v>
       </c>
-      <c r="B51" s="575" t="s">
+      <c r="B51" s="573" t="s">
         <v>271</v>
       </c>
       <c r="C51" s="37" t="s">
@@ -23848,8 +23848,8 @@
       </c>
     </row>
     <row r="52" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A52" s="574"/>
-      <c r="B52" s="576"/>
+      <c r="A52" s="571"/>
+      <c r="B52" s="574"/>
       <c r="C52" s="11" t="s">
         <v>272</v>
       </c>
@@ -23900,8 +23900,8 @@
       </c>
     </row>
     <row r="53" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A53" s="574"/>
-      <c r="B53" s="576"/>
+      <c r="A53" s="571"/>
+      <c r="B53" s="574"/>
       <c r="C53" s="11" t="s">
         <v>273</v>
       </c>
@@ -23952,8 +23952,8 @@
       </c>
     </row>
     <row r="54" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="574"/>
-      <c r="B54" s="576" t="s">
+      <c r="A54" s="571"/>
+      <c r="B54" s="574" t="s">
         <v>274</v>
       </c>
       <c r="C54" s="11" t="s">
@@ -24006,8 +24006,8 @@
       </c>
     </row>
     <row r="55" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A55" s="574"/>
-      <c r="B55" s="576"/>
+      <c r="A55" s="571"/>
+      <c r="B55" s="574"/>
       <c r="C55" s="11" t="s">
         <v>272</v>
       </c>
@@ -24058,8 +24058,8 @@
       </c>
     </row>
     <row r="56" spans="1:18" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="577"/>
-      <c r="B56" s="576"/>
+      <c r="A56" s="572"/>
+      <c r="B56" s="574"/>
       <c r="C56" s="11" t="s">
         <v>273</v>
       </c>
@@ -24111,6 +24111,25 @@
     </row>
   </sheetData>
   <mergeCells count="28">
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A3:A8"/>
+    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="A9:A14"/>
+    <mergeCell ref="B9:B11"/>
+    <mergeCell ref="B12:B14"/>
+    <mergeCell ref="A15:A20"/>
+    <mergeCell ref="B15:B17"/>
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="A21:A26"/>
+    <mergeCell ref="B21:B23"/>
+    <mergeCell ref="B24:B26"/>
+    <mergeCell ref="A27:A32"/>
+    <mergeCell ref="B27:B29"/>
+    <mergeCell ref="B30:B32"/>
+    <mergeCell ref="A33:A38"/>
+    <mergeCell ref="B33:B35"/>
+    <mergeCell ref="B36:B38"/>
     <mergeCell ref="A51:A56"/>
     <mergeCell ref="B51:B53"/>
     <mergeCell ref="B54:B56"/>
@@ -24120,25 +24139,6 @@
     <mergeCell ref="A45:A50"/>
     <mergeCell ref="B45:B47"/>
     <mergeCell ref="B48:B50"/>
-    <mergeCell ref="A27:A32"/>
-    <mergeCell ref="B27:B29"/>
-    <mergeCell ref="B30:B32"/>
-    <mergeCell ref="A33:A38"/>
-    <mergeCell ref="B33:B35"/>
-    <mergeCell ref="B36:B38"/>
-    <mergeCell ref="A15:A20"/>
-    <mergeCell ref="B15:B17"/>
-    <mergeCell ref="B18:B20"/>
-    <mergeCell ref="A21:A26"/>
-    <mergeCell ref="B21:B23"/>
-    <mergeCell ref="B24:B26"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A3:A8"/>
-    <mergeCell ref="B3:B5"/>
-    <mergeCell ref="B6:B8"/>
-    <mergeCell ref="A9:A14"/>
-    <mergeCell ref="B9:B11"/>
-    <mergeCell ref="B12:B14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -56700,10 +56700,10 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="60" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="B3" s="61" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C3" s="354">
         <v>64.536322439436617</v>
@@ -56748,7 +56748,7 @@
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="60"/>
       <c r="B4" s="61" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="C4" s="354" cm="1">
         <f t="array" ref="C4:O4">(25/30)*MI_2018!C4:O4+(5/30)*MI_2018!C5:O5</f>
@@ -56840,7 +56840,7 @@
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="60"/>
       <c r="B6" s="61" t="s">
-        <v>576</v>
+        <v>581</v>
       </c>
       <c r="C6" s="354">
         <v>53.747727971830976</v>
@@ -56884,10 +56884,10 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="60" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="B7" s="61" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C7" s="354">
         <v>51.236411047826117</v>
@@ -56932,7 +56932,7 @@
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" s="60"/>
       <c r="B8" s="61" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="C8" s="354" cm="1">
         <f t="array" ref="C8:O8">(25/30)*MI_2018!C8:O8+(5/30)*MI_2018!C9:O9</f>
@@ -57024,7 +57024,7 @@
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="60"/>
       <c r="B10" s="61" t="s">
-        <v>576</v>
+        <v>581</v>
       </c>
       <c r="C10" s="354">
         <v>54.810216828985524</v>
@@ -57071,7 +57071,7 @@
         <v>400</v>
       </c>
       <c r="B11" s="61" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C11" s="354">
         <v>46.466515152747249</v>
@@ -57116,7 +57116,7 @@
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="60"/>
       <c r="B12" s="61" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="C12" s="354" cm="1">
         <f t="array" ref="C12:O12">(25/30)*MI_2018!C12:O12+(5/30)*MI_2018!C13:O13</f>
@@ -57208,7 +57208,7 @@
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="60"/>
       <c r="B14" s="61" t="s">
-        <v>576</v>
+        <v>581</v>
       </c>
       <c r="C14" s="354">
         <v>48.035462363736258</v>
@@ -57252,10 +57252,10 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="60" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="B15" s="61" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C15" s="354">
         <v>63.247573617468966</v>
@@ -57300,7 +57300,7 @@
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" s="60"/>
       <c r="B16" s="61" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="C16" s="354" cm="1">
         <f t="array" ref="C16:O16">(25/30)*MI_2018!C16:O16+(5/30)*MI_2018!C17:O17</f>
@@ -57392,7 +57392,7 @@
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" s="60"/>
       <c r="B18" s="61" t="s">
-        <v>576</v>
+        <v>581</v>
       </c>
       <c r="C18" s="354">
         <v>78.130278452675611</v>
@@ -57439,7 +57439,7 @@
         <v>402</v>
       </c>
       <c r="B19" s="61" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C19" s="354">
         <v>73.961058518555888</v>
@@ -57484,7 +57484,7 @@
     <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" s="60"/>
       <c r="B20" s="61" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="C20" s="354" cm="1">
         <f t="array" ref="C20:O20">(25/30)*MI_2018!C20:O20+(5/30)*MI_2018!C21:O21</f>
@@ -57576,7 +57576,7 @@
     <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22" s="60"/>
       <c r="B22" s="61" t="s">
-        <v>576</v>
+        <v>581</v>
       </c>
       <c r="C22" s="354">
         <v>88.364030628762535</v>
@@ -57623,7 +57623,7 @@
         <v>403</v>
       </c>
       <c r="B23" s="61" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C23" s="354">
         <v>92.106593835443078</v>
@@ -57668,7 +57668,7 @@
     <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24" s="60"/>
       <c r="B24" s="61" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="C24" s="354" cm="1">
         <f t="array" ref="C24:O24">(25/30)*MI_2018!C24:O24+(5/30)*MI_2018!C25:O25</f>
@@ -57760,7 +57760,7 @@
     <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26" s="60"/>
       <c r="B26" s="61" t="s">
-        <v>576</v>
+        <v>581</v>
       </c>
       <c r="C26" s="354">
         <v>80.171314617411696</v>
@@ -57807,7 +57807,7 @@
         <v>404</v>
       </c>
       <c r="B27" s="61" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C27" s="354">
         <v>76.371623519910798</v>
@@ -57852,7 +57852,7 @@
     <row r="28" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A28" s="60"/>
       <c r="B28" s="61" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="C28" s="354" cm="1">
         <f t="array" ref="C28:O28">(25/30)*MI_2018!C28:O28+(5/30)*MI_2018!C29:O29</f>
@@ -57944,7 +57944,7 @@
     <row r="30" spans="1:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A30" s="66"/>
       <c r="B30" s="61" t="s">
-        <v>576</v>
+        <v>581</v>
       </c>
       <c r="C30" s="354">
         <v>77.420896134762941</v>

</xml_diff>

<commit_message>
amendment to the building type rename
</commit_message>
<xml_diff>
--- a/data_input/MI_Buildings_Oorschot2023.xlsx
+++ b/data_input/MI_Buildings_Oorschot2023.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Mira/Documents/IE/REAL UTOPIAN HOUSING/Post-GrowthHousingScenarios/Code/housing-footprints/data_input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6A3E593-33EB-4540-B39B-01C96BD18665}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AEB5C0C-B410-C448-ADA9-0E521AE16BA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10660" yWindow="500" windowWidth="14940" windowHeight="15500" tabRatio="902" activeTab="2" xr2:uid="{501A363E-84AB-4328-B285-EDCE5CC29F1E}"/>
+    <workbookView xWindow="10660" yWindow="500" windowWidth="14940" windowHeight="15500" tabRatio="902" firstSheet="8" activeTab="5" xr2:uid="{501A363E-84AB-4328-B285-EDCE5CC29F1E}"/>
   </bookViews>
   <sheets>
     <sheet name="Content" sheetId="24" r:id="rId1"/>
@@ -105,7 +105,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2878" uniqueCount="582">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2878" uniqueCount="581">
   <si>
     <t>aluminium, wrought alloy | treatment of aluminium scrap, post-consumer, prepared for recycling, at remelter | RER | kilogram | cutoff38 - Janneke</t>
   </si>
@@ -2145,16 +2145,13 @@
     <t>1946-1974</t>
   </si>
   <si>
-    <t>detached (vrijstaand)</t>
+    <t>2006-2022</t>
   </si>
   <si>
-    <t>row house (tussenwoning)</t>
+    <t>detached</t>
   </si>
   <si>
-    <t>multiple fam (meergezins)</t>
-  </si>
-  <si>
-    <t>2006-2022</t>
+    <t>multifamily</t>
   </si>
 </sst>
 </file>
@@ -4432,10 +4429,16 @@
     <xf numFmtId="0" fontId="57" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -4444,13 +4447,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -21200,11 +21197,11 @@
       </c>
     </row>
     <row r="2" spans="1:18" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="575">
+      <c r="A2" s="571">
         <v>2018</v>
       </c>
-      <c r="B2" s="576"/>
-      <c r="C2" s="576"/>
+      <c r="B2" s="572"/>
+      <c r="C2" s="572"/>
       <c r="D2" s="174">
         <v>1849352203.1438973</v>
       </c>
@@ -21248,10 +21245,10 @@
       <c r="R2" s="175"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A3" s="577" t="s">
+      <c r="A3" s="573" t="s">
         <v>235</v>
       </c>
-      <c r="B3" s="573" t="s">
+      <c r="B3" s="575" t="s">
         <v>271</v>
       </c>
       <c r="C3" s="37" t="s">
@@ -21304,8 +21301,8 @@
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A4" s="571"/>
-      <c r="B4" s="574"/>
+      <c r="A4" s="574"/>
+      <c r="B4" s="576"/>
       <c r="C4" s="11" t="s">
         <v>272</v>
       </c>
@@ -21356,8 +21353,8 @@
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A5" s="571"/>
-      <c r="B5" s="574"/>
+      <c r="A5" s="574"/>
+      <c r="B5" s="576"/>
       <c r="C5" s="11" t="s">
         <v>273</v>
       </c>
@@ -21408,8 +21405,8 @@
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A6" s="571"/>
-      <c r="B6" s="574" t="s">
+      <c r="A6" s="574"/>
+      <c r="B6" s="576" t="s">
         <v>274</v>
       </c>
       <c r="C6" s="11" t="s">
@@ -21462,8 +21459,8 @@
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A7" s="571"/>
-      <c r="B7" s="574"/>
+      <c r="A7" s="574"/>
+      <c r="B7" s="576"/>
       <c r="C7" s="11" t="s">
         <v>272</v>
       </c>
@@ -21514,8 +21511,8 @@
       </c>
     </row>
     <row r="8" spans="1:18" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="571"/>
-      <c r="B8" s="574"/>
+      <c r="A8" s="574"/>
+      <c r="B8" s="576"/>
       <c r="C8" s="11" t="s">
         <v>273</v>
       </c>
@@ -21566,10 +21563,10 @@
       </c>
     </row>
     <row r="9" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="571" t="s">
+      <c r="A9" s="574" t="s">
         <v>275</v>
       </c>
-      <c r="B9" s="573" t="s">
+      <c r="B9" s="575" t="s">
         <v>271</v>
       </c>
       <c r="C9" s="37" t="s">
@@ -21622,8 +21619,8 @@
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A10" s="571"/>
-      <c r="B10" s="574"/>
+      <c r="A10" s="574"/>
+      <c r="B10" s="576"/>
       <c r="C10" s="11" t="s">
         <v>272</v>
       </c>
@@ -21674,8 +21671,8 @@
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A11" s="571"/>
-      <c r="B11" s="574"/>
+      <c r="A11" s="574"/>
+      <c r="B11" s="576"/>
       <c r="C11" s="11" t="s">
         <v>273</v>
       </c>
@@ -21726,8 +21723,8 @@
       </c>
     </row>
     <row r="12" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="571"/>
-      <c r="B12" s="574" t="s">
+      <c r="A12" s="574"/>
+      <c r="B12" s="576" t="s">
         <v>274</v>
       </c>
       <c r="C12" s="11" t="s">
@@ -21780,8 +21777,8 @@
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A13" s="571"/>
-      <c r="B13" s="574"/>
+      <c r="A13" s="574"/>
+      <c r="B13" s="576"/>
       <c r="C13" s="11" t="s">
         <v>272</v>
       </c>
@@ -21832,8 +21829,8 @@
       </c>
     </row>
     <row r="14" spans="1:18" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="571"/>
-      <c r="B14" s="574"/>
+      <c r="A14" s="574"/>
+      <c r="B14" s="576"/>
       <c r="C14" s="11" t="s">
         <v>273</v>
       </c>
@@ -21884,10 +21881,10 @@
       </c>
     </row>
     <row r="15" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="571" t="s">
+      <c r="A15" s="574" t="s">
         <v>276</v>
       </c>
-      <c r="B15" s="573" t="s">
+      <c r="B15" s="575" t="s">
         <v>271</v>
       </c>
       <c r="C15" s="37" t="s">
@@ -21940,8 +21937,8 @@
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A16" s="571"/>
-      <c r="B16" s="574"/>
+      <c r="A16" s="574"/>
+      <c r="B16" s="576"/>
       <c r="C16" s="11" t="s">
         <v>272</v>
       </c>
@@ -21992,8 +21989,8 @@
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A17" s="571"/>
-      <c r="B17" s="574"/>
+      <c r="A17" s="574"/>
+      <c r="B17" s="576"/>
       <c r="C17" s="11" t="s">
         <v>273</v>
       </c>
@@ -22044,8 +22041,8 @@
       </c>
     </row>
     <row r="18" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="571"/>
-      <c r="B18" s="574" t="s">
+      <c r="A18" s="574"/>
+      <c r="B18" s="576" t="s">
         <v>274</v>
       </c>
       <c r="C18" s="11" t="s">
@@ -22098,8 +22095,8 @@
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A19" s="571"/>
-      <c r="B19" s="574"/>
+      <c r="A19" s="574"/>
+      <c r="B19" s="576"/>
       <c r="C19" s="11" t="s">
         <v>272</v>
       </c>
@@ -22150,8 +22147,8 @@
       </c>
     </row>
     <row r="20" spans="1:18" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="571"/>
-      <c r="B20" s="574"/>
+      <c r="A20" s="574"/>
+      <c r="B20" s="576"/>
       <c r="C20" s="11" t="s">
         <v>273</v>
       </c>
@@ -22202,10 +22199,10 @@
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A21" s="571" t="s">
+      <c r="A21" s="574" t="s">
         <v>236</v>
       </c>
-      <c r="B21" s="573" t="s">
+      <c r="B21" s="575" t="s">
         <v>271</v>
       </c>
       <c r="C21" s="37" t="s">
@@ -22258,8 +22255,8 @@
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A22" s="571"/>
-      <c r="B22" s="574"/>
+      <c r="A22" s="574"/>
+      <c r="B22" s="576"/>
       <c r="C22" s="11" t="s">
         <v>272</v>
       </c>
@@ -22310,8 +22307,8 @@
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A23" s="571"/>
-      <c r="B23" s="574"/>
+      <c r="A23" s="574"/>
+      <c r="B23" s="576"/>
       <c r="C23" s="11" t="s">
         <v>273</v>
       </c>
@@ -22362,8 +22359,8 @@
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A24" s="571"/>
-      <c r="B24" s="574" t="s">
+      <c r="A24" s="574"/>
+      <c r="B24" s="576" t="s">
         <v>274</v>
       </c>
       <c r="C24" s="11" t="s">
@@ -22416,8 +22413,8 @@
       </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A25" s="571"/>
-      <c r="B25" s="574"/>
+      <c r="A25" s="574"/>
+      <c r="B25" s="576"/>
       <c r="C25" s="11" t="s">
         <v>272</v>
       </c>
@@ -22468,8 +22465,8 @@
       </c>
     </row>
     <row r="26" spans="1:18" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="571"/>
-      <c r="B26" s="574"/>
+      <c r="A26" s="574"/>
+      <c r="B26" s="576"/>
       <c r="C26" s="11" t="s">
         <v>273</v>
       </c>
@@ -22520,10 +22517,10 @@
       </c>
     </row>
     <row r="27" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="571" t="s">
+      <c r="A27" s="574" t="s">
         <v>277</v>
       </c>
-      <c r="B27" s="573" t="s">
+      <c r="B27" s="575" t="s">
         <v>271</v>
       </c>
       <c r="C27" s="37" t="s">
@@ -22576,8 +22573,8 @@
       </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A28" s="571"/>
-      <c r="B28" s="574"/>
+      <c r="A28" s="574"/>
+      <c r="B28" s="576"/>
       <c r="C28" s="11" t="s">
         <v>272</v>
       </c>
@@ -22628,8 +22625,8 @@
       </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A29" s="571"/>
-      <c r="B29" s="574"/>
+      <c r="A29" s="574"/>
+      <c r="B29" s="576"/>
       <c r="C29" s="11" t="s">
         <v>273</v>
       </c>
@@ -22680,8 +22677,8 @@
       </c>
     </row>
     <row r="30" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="571"/>
-      <c r="B30" s="574" t="s">
+      <c r="A30" s="574"/>
+      <c r="B30" s="576" t="s">
         <v>274</v>
       </c>
       <c r="C30" s="11" t="s">
@@ -22734,8 +22731,8 @@
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A31" s="571"/>
-      <c r="B31" s="574"/>
+      <c r="A31" s="574"/>
+      <c r="B31" s="576"/>
       <c r="C31" s="11" t="s">
         <v>272</v>
       </c>
@@ -22786,8 +22783,8 @@
       </c>
     </row>
     <row r="32" spans="1:18" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="571"/>
-      <c r="B32" s="574"/>
+      <c r="A32" s="574"/>
+      <c r="B32" s="576"/>
       <c r="C32" s="11" t="s">
         <v>273</v>
       </c>
@@ -22838,10 +22835,10 @@
       </c>
     </row>
     <row r="33" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="571" t="s">
+      <c r="A33" s="574" t="s">
         <v>278</v>
       </c>
-      <c r="B33" s="573" t="s">
+      <c r="B33" s="575" t="s">
         <v>271</v>
       </c>
       <c r="C33" s="37" t="s">
@@ -22894,8 +22891,8 @@
       </c>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A34" s="571"/>
-      <c r="B34" s="574"/>
+      <c r="A34" s="574"/>
+      <c r="B34" s="576"/>
       <c r="C34" s="11" t="s">
         <v>272</v>
       </c>
@@ -22946,8 +22943,8 @@
       </c>
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A35" s="571"/>
-      <c r="B35" s="574"/>
+      <c r="A35" s="574"/>
+      <c r="B35" s="576"/>
       <c r="C35" s="11" t="s">
         <v>273</v>
       </c>
@@ -22998,8 +22995,8 @@
       </c>
     </row>
     <row r="36" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="571"/>
-      <c r="B36" s="574" t="s">
+      <c r="A36" s="574"/>
+      <c r="B36" s="576" t="s">
         <v>274</v>
       </c>
       <c r="C36" s="11" t="s">
@@ -23052,8 +23049,8 @@
       </c>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A37" s="571"/>
-      <c r="B37" s="574"/>
+      <c r="A37" s="574"/>
+      <c r="B37" s="576"/>
       <c r="C37" s="11" t="s">
         <v>272</v>
       </c>
@@ -23104,8 +23101,8 @@
       </c>
     </row>
     <row r="38" spans="1:18" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="571"/>
-      <c r="B38" s="574"/>
+      <c r="A38" s="574"/>
+      <c r="B38" s="576"/>
       <c r="C38" s="11" t="s">
         <v>273</v>
       </c>
@@ -23156,10 +23153,10 @@
       </c>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A39" s="571" t="s">
+      <c r="A39" s="574" t="s">
         <v>241</v>
       </c>
-      <c r="B39" s="573" t="s">
+      <c r="B39" s="575" t="s">
         <v>271</v>
       </c>
       <c r="C39" s="37" t="s">
@@ -23212,8 +23209,8 @@
       </c>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A40" s="571"/>
-      <c r="B40" s="574"/>
+      <c r="A40" s="574"/>
+      <c r="B40" s="576"/>
       <c r="C40" s="11" t="s">
         <v>272</v>
       </c>
@@ -23264,8 +23261,8 @@
       </c>
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A41" s="571"/>
-      <c r="B41" s="574"/>
+      <c r="A41" s="574"/>
+      <c r="B41" s="576"/>
       <c r="C41" s="11" t="s">
         <v>273</v>
       </c>
@@ -23316,8 +23313,8 @@
       </c>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A42" s="571"/>
-      <c r="B42" s="574" t="s">
+      <c r="A42" s="574"/>
+      <c r="B42" s="576" t="s">
         <v>274</v>
       </c>
       <c r="C42" s="11" t="s">
@@ -23370,8 +23367,8 @@
       </c>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A43" s="571"/>
-      <c r="B43" s="574"/>
+      <c r="A43" s="574"/>
+      <c r="B43" s="576"/>
       <c r="C43" s="11" t="s">
         <v>272</v>
       </c>
@@ -23422,8 +23419,8 @@
       </c>
     </row>
     <row r="44" spans="1:18" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="571"/>
-      <c r="B44" s="574"/>
+      <c r="A44" s="574"/>
+      <c r="B44" s="576"/>
       <c r="C44" s="11" t="s">
         <v>273</v>
       </c>
@@ -23474,10 +23471,10 @@
       </c>
     </row>
     <row r="45" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="571" t="s">
+      <c r="A45" s="574" t="s">
         <v>393</v>
       </c>
-      <c r="B45" s="573" t="s">
+      <c r="B45" s="575" t="s">
         <v>271</v>
       </c>
       <c r="C45" s="37" t="s">
@@ -23530,8 +23527,8 @@
       </c>
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A46" s="571"/>
-      <c r="B46" s="574"/>
+      <c r="A46" s="574"/>
+      <c r="B46" s="576"/>
       <c r="C46" s="11" t="s">
         <v>272</v>
       </c>
@@ -23582,8 +23579,8 @@
       </c>
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A47" s="571"/>
-      <c r="B47" s="574"/>
+      <c r="A47" s="574"/>
+      <c r="B47" s="576"/>
       <c r="C47" s="11" t="s">
         <v>273</v>
       </c>
@@ -23634,8 +23631,8 @@
       </c>
     </row>
     <row r="48" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="571"/>
-      <c r="B48" s="574" t="s">
+      <c r="A48" s="574"/>
+      <c r="B48" s="576" t="s">
         <v>274</v>
       </c>
       <c r="C48" s="11" t="s">
@@ -23688,8 +23685,8 @@
       </c>
     </row>
     <row r="49" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A49" s="571"/>
-      <c r="B49" s="574"/>
+      <c r="A49" s="574"/>
+      <c r="B49" s="576"/>
       <c r="C49" s="11" t="s">
         <v>272</v>
       </c>
@@ -23740,8 +23737,8 @@
       </c>
     </row>
     <row r="50" spans="1:18" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="571"/>
-      <c r="B50" s="574"/>
+      <c r="A50" s="574"/>
+      <c r="B50" s="576"/>
       <c r="C50" s="11" t="s">
         <v>273</v>
       </c>
@@ -23792,10 +23789,10 @@
       </c>
     </row>
     <row r="51" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="571" t="s">
+      <c r="A51" s="574" t="s">
         <v>394</v>
       </c>
-      <c r="B51" s="573" t="s">
+      <c r="B51" s="575" t="s">
         <v>271</v>
       </c>
       <c r="C51" s="37" t="s">
@@ -23848,8 +23845,8 @@
       </c>
     </row>
     <row r="52" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A52" s="571"/>
-      <c r="B52" s="574"/>
+      <c r="A52" s="574"/>
+      <c r="B52" s="576"/>
       <c r="C52" s="11" t="s">
         <v>272</v>
       </c>
@@ -23900,8 +23897,8 @@
       </c>
     </row>
     <row r="53" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A53" s="571"/>
-      <c r="B53" s="574"/>
+      <c r="A53" s="574"/>
+      <c r="B53" s="576"/>
       <c r="C53" s="11" t="s">
         <v>273</v>
       </c>
@@ -23952,8 +23949,8 @@
       </c>
     </row>
     <row r="54" spans="1:18" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="571"/>
-      <c r="B54" s="574" t="s">
+      <c r="A54" s="574"/>
+      <c r="B54" s="576" t="s">
         <v>274</v>
       </c>
       <c r="C54" s="11" t="s">
@@ -24006,8 +24003,8 @@
       </c>
     </row>
     <row r="55" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A55" s="571"/>
-      <c r="B55" s="574"/>
+      <c r="A55" s="574"/>
+      <c r="B55" s="576"/>
       <c r="C55" s="11" t="s">
         <v>272</v>
       </c>
@@ -24058,8 +24055,8 @@
       </c>
     </row>
     <row r="56" spans="1:18" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="572"/>
-      <c r="B56" s="574"/>
+      <c r="A56" s="577"/>
+      <c r="B56" s="576"/>
       <c r="C56" s="11" t="s">
         <v>273</v>
       </c>
@@ -24111,25 +24108,6 @@
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A3:A8"/>
-    <mergeCell ref="B3:B5"/>
-    <mergeCell ref="B6:B8"/>
-    <mergeCell ref="A9:A14"/>
-    <mergeCell ref="B9:B11"/>
-    <mergeCell ref="B12:B14"/>
-    <mergeCell ref="A15:A20"/>
-    <mergeCell ref="B15:B17"/>
-    <mergeCell ref="B18:B20"/>
-    <mergeCell ref="A21:A26"/>
-    <mergeCell ref="B21:B23"/>
-    <mergeCell ref="B24:B26"/>
-    <mergeCell ref="A27:A32"/>
-    <mergeCell ref="B27:B29"/>
-    <mergeCell ref="B30:B32"/>
-    <mergeCell ref="A33:A38"/>
-    <mergeCell ref="B33:B35"/>
-    <mergeCell ref="B36:B38"/>
     <mergeCell ref="A51:A56"/>
     <mergeCell ref="B51:B53"/>
     <mergeCell ref="B54:B56"/>
@@ -24139,6 +24117,25 @@
     <mergeCell ref="A45:A50"/>
     <mergeCell ref="B45:B47"/>
     <mergeCell ref="B48:B50"/>
+    <mergeCell ref="A27:A32"/>
+    <mergeCell ref="B27:B29"/>
+    <mergeCell ref="B30:B32"/>
+    <mergeCell ref="A33:A38"/>
+    <mergeCell ref="B33:B35"/>
+    <mergeCell ref="B36:B38"/>
+    <mergeCell ref="A15:A20"/>
+    <mergeCell ref="B15:B17"/>
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="A21:A26"/>
+    <mergeCell ref="B21:B23"/>
+    <mergeCell ref="B24:B26"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A3:A8"/>
+    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="A9:A14"/>
+    <mergeCell ref="B9:B11"/>
+    <mergeCell ref="B12:B14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -56700,7 +56697,7 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="60" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="B3" s="61" t="s">
         <v>576</v>
@@ -56840,7 +56837,7 @@
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="60"/>
       <c r="B6" s="61" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="C6" s="354">
         <v>53.747727971830976</v>
@@ -56884,7 +56881,7 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="60" t="s">
-        <v>579</v>
+        <v>399</v>
       </c>
       <c r="B7" s="61" t="s">
         <v>576</v>
@@ -57024,7 +57021,7 @@
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="60"/>
       <c r="B10" s="61" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="C10" s="354">
         <v>54.810216828985524</v>
@@ -57208,7 +57205,7 @@
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="60"/>
       <c r="B14" s="61" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="C14" s="354">
         <v>48.035462363736258</v>
@@ -57392,7 +57389,7 @@
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" s="60"/>
       <c r="B18" s="61" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="C18" s="354">
         <v>78.130278452675611</v>
@@ -57576,7 +57573,7 @@
     <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22" s="60"/>
       <c r="B22" s="61" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="C22" s="354">
         <v>88.364030628762535</v>
@@ -57760,7 +57757,7 @@
     <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26" s="60"/>
       <c r="B26" s="61" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="C26" s="354">
         <v>80.171314617411696</v>
@@ -57944,7 +57941,7 @@
     <row r="30" spans="1:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A30" s="66"/>
       <c r="B30" s="61" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="C30" s="354">
         <v>77.420896134762941</v>

</xml_diff>